<commit_message>
feat: expand mobile catalogs and emergency service requests
</commit_message>
<xml_diff>
--- a/صلاحيات_النظام.xlsx
+++ b/صلاحيات_النظام.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="كل الصلاحيات" sheetId="1" r:id="R1685527c1cea4dda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ملخص حسب الوحدة" sheetId="2" r:id="R73915772de0346a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اختبار الأدوار" sheetId="3" r:id="R39f5e5b0b41c4d6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اعتماد الزبائن" sheetId="4" r:id="R20bf0a86f71541c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="كل الصلاحيات" sheetId="1" r:id="Rb88743d3308349c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ملخص حسب الوحدة" sheetId="2" r:id="R37c09b18b5974d6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اختبار الأدوار" sheetId="3" r:id="R5f5627e2b7ba4a37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اعتماد الزبائن" sheetId="4" r:id="R65ca32fa3558422c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,7 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="15">
+  <x:fonts count="17">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -93,8 +93,19 @@
       <x:color rgb="FF006100"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF008000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF008000"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="34">
+  <x:fills count="35">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -261,6 +272,11 @@
         <x:fgColor rgb="FFC6EFCE"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -296,7 +312,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="96">
+  <x:cellXfs count="101">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -545,6 +561,15 @@
     <x:xf numFmtId="0" fontId="14" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -9833,6 +9858,46 @@
         <x:v>إضافة 2026-07-27: تعيين موظف مؤهل أو نقل ملكية الاسم إلى الفرع. مستقلة عن candidates.edit.</x:v>
       </x:c>
     </x:row>
+    <x:row r="151">
+      <x:c r="A151" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="B151"/>
+      <x:c r="C151" t="str">
+        <x:v>طلبات الخدمة والصيانة</x:v>
+      </x:c>
+      <x:c r="D151" t="str">
+        <x:v>service_requests</x:v>
+      </x:c>
+      <x:c r="E151" t="str">
+        <x:v>service_requests</x:v>
+      </x:c>
+      <x:c r="F151" t="str">
+        <x:v>override_active_emergency</x:v>
+      </x:c>
+      <x:c r="G151" t="str">
+        <x:v>فتح مهمة صيانة طارئة مستقلة رغم وجود مهمة نشطة</x:v>
+      </x:c>
+      <x:c r="H151" t="str">
+        <x:v>service_requests.override_active_emergency</x:v>
+      </x:c>
+      <x:c r="I151" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J151" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="K151" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L151"/>
+      <x:c r="M151" s="98" t="str">
+        <x:v>تمت الإضافة</x:v>
+      </x:c>
+      <x:c r="N151" s="98" t="str">
+        <x:v>إضافة جديدة: استثناء موثق لفتح مهمة طارئة ثانية على الجهاز نفسه. GLOBAL فقط ويلزم سبب من القائمة النظامية.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9966,7 +10031,7 @@
         </x:is>
       </x:c>
       <x:c r="C8" s="29" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -10196,7 +10261,7 @@
       </x:c>
       <x:c r="B24"/>
       <x:c r="C24" t="n">
-        <x:v>149</x:v>
+        <x:v>150</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -16986,6 +17051,40 @@
         <x:v>إضافة 2026-07-27: مدير الفرع ومدير الشركة ضمن BRANCH؛ السوبر أدمن مسار التجاوز الصريح.</x:v>
       </x:c>
     </x:row>
+    <x:row r="143">
+      <x:c r="A143" t="n">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="B143"/>
+      <x:c r="C143" t="str">
+        <x:v>service_requests.override_active_emergency</x:v>
+      </x:c>
+      <x:c r="D143" t="str">
+        <x:v>طلبات الخدمة والصيانة</x:v>
+      </x:c>
+      <x:c r="E143" t="str">
+        <x:v>override_active_emergency</x:v>
+      </x:c>
+      <x:c r="F143" s="100" t="str">
+        <x:v>تمت الإضافة</x:v>
+      </x:c>
+      <x:c r="G143" s="100"/>
+      <x:c r="H143" s="100"/>
+      <x:c r="I143" s="100"/>
+      <x:c r="J143" s="100"/>
+      <x:c r="K143" s="100"/>
+      <x:c r="L143" s="100"/>
+      <x:c r="M143" s="100" t="str">
+        <x:v>لا تُمنح افتراضياً. GLOBAL فقط وبقرار إداري صريح.</x:v>
+      </x:c>
+      <x:c r="N143"/>
+      <x:c r="O143"/>
+      <x:c r="P143"/>
+      <x:c r="Q143"/>
+      <x:c r="R143"/>
+      <x:c r="S143"/>
+      <x:c r="T143"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat: expand mobile service request workflows
</commit_message>
<xml_diff>
--- a/صلاحيات_النظام.xlsx
+++ b/صلاحيات_النظام.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="كل الصلاحيات" sheetId="1" r:id="R9159ecccbcf74a31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ملخص حسب الوحدة" sheetId="2" r:id="R3b22dcdfb16a43e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اختبار الأدوار" sheetId="3" r:id="R2a6b69d48d284179"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اعتماد الزبائن" sheetId="4" r:id="Rec2433b277834833"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="كل الصلاحيات" sheetId="1" r:id="Ra68476b2bf65462c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ملخص حسب الوحدة" sheetId="2" r:id="R098bec007bd54e06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اختبار الأدوار" sheetId="3" r:id="Ra14a408661e64aa7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اعتماد الزبائن" sheetId="4" r:id="Raafa0d347e7c45e5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -117,7 +117,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="41">
+  <x:fills count="42">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -319,6 +319,11 @@
         <x:fgColor rgb="FFC6EFCE"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC6EFCE"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -354,7 +359,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="124">
+  <x:cellXfs count="126">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -649,6 +654,8 @@
     <x:xf numFmtId="0" fontId="14" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -10657,6 +10664,206 @@
         <x:v>صلاحية مركزية بنطاق GLOBAL فقط؛ لا يعتمد القرار على فرع الطلب.</x:v>
       </x:c>
     </x:row>
+    <x:row r="169">
+      <x:c r="A169" s="125" t="n">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="B169" s="125"/>
+      <x:c r="C169" s="125" t="str">
+        <x:v>طلبات ترخيص الوكلاء</x:v>
+      </x:c>
+      <x:c r="D169" s="125" t="str">
+        <x:v>agent_license</x:v>
+      </x:c>
+      <x:c r="E169" s="125" t="str">
+        <x:v>service_requests</x:v>
+      </x:c>
+      <x:c r="F169" s="125" t="str">
+        <x:v>view</x:v>
+      </x:c>
+      <x:c r="G169" s="125" t="str">
+        <x:v>عرض طلبات ترخيص الوكلاء</x:v>
+      </x:c>
+      <x:c r="H169" s="125" t="str">
+        <x:v>agent_license.view</x:v>
+      </x:c>
+      <x:c r="I169" s="125" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J169" s="125" t="n">
+        <x:v>297</x:v>
+      </x:c>
+      <x:c r="K169" s="125" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L169" s="125"/>
+      <x:c r="M169" s="125" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="N169" s="125" t="str">
+        <x:v>صلاحية مركزية بنطاق GLOBAL فقط؛ لا يعتمد القرار على فرع الطلب.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170">
+      <x:c r="A170" s="125" t="n">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="B170" s="125"/>
+      <x:c r="C170" s="125" t="str">
+        <x:v>طلبات ترخيص الوكلاء</x:v>
+      </x:c>
+      <x:c r="D170" s="125" t="str">
+        <x:v>agent_license</x:v>
+      </x:c>
+      <x:c r="E170" s="125" t="str">
+        <x:v>service_requests</x:v>
+      </x:c>
+      <x:c r="F170" s="125" t="str">
+        <x:v>review</x:v>
+      </x:c>
+      <x:c r="G170" s="125" t="str">
+        <x:v>مراجعة وربط طلبات ترخيص الوكلاء</x:v>
+      </x:c>
+      <x:c r="H170" s="125" t="str">
+        <x:v>agent_license.review</x:v>
+      </x:c>
+      <x:c r="I170" s="125" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J170" s="125" t="n">
+        <x:v>298</x:v>
+      </x:c>
+      <x:c r="K170" s="125" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L170" s="125"/>
+      <x:c r="M170" s="125" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="N170" s="125" t="str">
+        <x:v>تسمح بالتولي والمطابقة والربط الاختياري بزبون؛ GLOBAL فقط.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171">
+      <x:c r="A171" s="125" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="B171" s="125"/>
+      <x:c r="C171" s="125" t="str">
+        <x:v>طلبات ترخيص الوكلاء</x:v>
+      </x:c>
+      <x:c r="D171" s="125" t="str">
+        <x:v>agent_license</x:v>
+      </x:c>
+      <x:c r="E171" s="125" t="str">
+        <x:v>service_requests</x:v>
+      </x:c>
+      <x:c r="F171" s="125" t="str">
+        <x:v>decide</x:v>
+      </x:c>
+      <x:c r="G171" s="125" t="str">
+        <x:v>حسم طلبات ترخيص الوكلاء</x:v>
+      </x:c>
+      <x:c r="H171" s="125" t="str">
+        <x:v>agent_license.decide</x:v>
+      </x:c>
+      <x:c r="I171" s="125" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J171" s="125" t="n">
+        <x:v>299</x:v>
+      </x:c>
+      <x:c r="K171" s="125" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L171" s="125"/>
+      <x:c r="M171" s="125" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="N171" s="125" t="str">
+        <x:v>تسمح بالموافقة إلى completed أو الرفض أو الإلغاء؛ لا إعادة فتح ولا حل محايد ظاهر.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" s="125" t="n">
+        <x:v>171</x:v>
+      </x:c>
+      <x:c r="B172" s="125"/>
+      <x:c r="C172" s="125" t="str">
+        <x:v>طلبات ترخيص الوكلاء</x:v>
+      </x:c>
+      <x:c r="D172" s="125" t="str">
+        <x:v>agent_license</x:v>
+      </x:c>
+      <x:c r="E172" s="125" t="str">
+        <x:v>service_requests</x:v>
+      </x:c>
+      <x:c r="F172" s="125" t="str">
+        <x:v>resolve_escalation</x:v>
+      </x:c>
+      <x:c r="G172" s="125" t="str">
+        <x:v>فك تصعيد طلبات ترخيص الوكلاء</x:v>
+      </x:c>
+      <x:c r="H172" s="125" t="str">
+        <x:v>agent_license.resolve_escalation</x:v>
+      </x:c>
+      <x:c r="I172" s="125" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J172" s="125" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="K172" s="125" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L172" s="125"/>
+      <x:c r="M172" s="125" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="N172" s="125" t="str">
+        <x:v>صلاحية مركزية بنطاق GLOBAL فقط مع مسار super-admin الصريح.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173">
+      <x:c r="A173" s="125" t="n">
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="B173" s="125"/>
+      <x:c r="C173" s="125" t="str">
+        <x:v>طلبات ترخيص الوكلاء</x:v>
+      </x:c>
+      <x:c r="D173" s="125" t="str">
+        <x:v>agent_license</x:v>
+      </x:c>
+      <x:c r="E173" s="125" t="str">
+        <x:v>service_requests</x:v>
+      </x:c>
+      <x:c r="F173" s="125" t="str">
+        <x:v>archive</x:v>
+      </x:c>
+      <x:c r="G173" s="125" t="str">
+        <x:v>أرشفة طلبات ترخيص الوكلاء</x:v>
+      </x:c>
+      <x:c r="H173" s="125" t="str">
+        <x:v>agent_license.archive</x:v>
+      </x:c>
+      <x:c r="I173" s="125" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J173" s="125" t="n">
+        <x:v>301</x:v>
+      </x:c>
+      <x:c r="K173" s="125" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L173" s="125"/>
+      <x:c r="M173" s="125" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="N173" s="125" t="str">
+        <x:v>الأرشفة لا تغير نتيجة الطلب؛ صلاحية مركزية بنطاق GLOBAL فقط.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11038,11 +11245,33 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" t="str">
+        <x:v>طلبات ترشيح الأسماء</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>name_nomination</x:v>
+      </x:c>
+      <x:c r="C26" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="125" t="str">
+        <x:v>طلبات ترخيص الوكلاء</x:v>
+      </x:c>
+      <x:c r="B27" s="125" t="str">
+        <x:v>agent_license</x:v>
+      </x:c>
+      <x:c r="C27" s="125" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
         <x:v>الإجمالي</x:v>
       </x:c>
-      <x:c r="B26"/>
-      <x:c r="C26" t="n">
-        <x:v>162</x:v>
+      <x:c r="B28"/>
+      <x:c r="C28" t="n">
+        <x:v>172</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -18298,6 +18527,186 @@
         <x:v>إضافة 2026-08-11: عام (كل الفروع) / الفرع. المنح تضبط من شاشة الأدوار؛ create فقط يبذر للأدوار التي تجمع صلاحية الاتصال وإنشاء طلب خدمة.</x:v>
       </x:c>
     </x:row>
+    <x:row r="156">
+      <x:c r="A156" s="125" t="n">
+        <x:v>155</x:v>
+      </x:c>
+      <x:c r="B156" s="125"/>
+      <x:c r="C156" s="125" t="str">
+        <x:v>agent_license.view</x:v>
+      </x:c>
+      <x:c r="D156" s="125" t="str">
+        <x:v>طلبات ترخيص الوكلاء</x:v>
+      </x:c>
+      <x:c r="E156" s="125" t="str">
+        <x:v>view</x:v>
+      </x:c>
+      <x:c r="F156" s="125" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G156" s="125"/>
+      <x:c r="H156" s="125"/>
+      <x:c r="I156" s="125"/>
+      <x:c r="J156" s="125"/>
+      <x:c r="K156" s="125"/>
+      <x:c r="L156" s="125"/>
+      <x:c r="M156" s="125" t="str">
+        <x:v>قرار حسب الدور</x:v>
+      </x:c>
+      <x:c r="N156" s="125"/>
+      <x:c r="O156" s="125"/>
+      <x:c r="P156" s="125"/>
+      <x:c r="Q156" s="125"/>
+      <x:c r="R156" s="125"/>
+      <x:c r="S156" s="125"/>
+      <x:c r="T156" s="125" t="str">
+        <x:v>إضافة 2026-08-12: عام (كل الفروع) فقط. المنح تضبط من شاشة الأدوار؛ لا يوجد منح تلقائي أو create داخلي.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157">
+      <x:c r="A157" s="125" t="n">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="B157" s="125"/>
+      <x:c r="C157" s="125" t="str">
+        <x:v>agent_license.review</x:v>
+      </x:c>
+      <x:c r="D157" s="125" t="str">
+        <x:v>طلبات ترخيص الوكلاء</x:v>
+      </x:c>
+      <x:c r="E157" s="125" t="str">
+        <x:v>review</x:v>
+      </x:c>
+      <x:c r="F157" s="125" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G157" s="125"/>
+      <x:c r="H157" s="125"/>
+      <x:c r="I157" s="125"/>
+      <x:c r="J157" s="125"/>
+      <x:c r="K157" s="125"/>
+      <x:c r="L157" s="125"/>
+      <x:c r="M157" s="125" t="str">
+        <x:v>قرار حسب الدور</x:v>
+      </x:c>
+      <x:c r="N157" s="125"/>
+      <x:c r="O157" s="125"/>
+      <x:c r="P157" s="125"/>
+      <x:c r="Q157" s="125"/>
+      <x:c r="R157" s="125"/>
+      <x:c r="S157" s="125"/>
+      <x:c r="T157" s="125" t="str">
+        <x:v>إضافة 2026-08-12: عام (كل الفروع) فقط. المنح تضبط من شاشة الأدوار؛ لا يوجد منح تلقائي أو create داخلي.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158">
+      <x:c r="A158" s="125" t="n">
+        <x:v>157</x:v>
+      </x:c>
+      <x:c r="B158" s="125"/>
+      <x:c r="C158" s="125" t="str">
+        <x:v>agent_license.decide</x:v>
+      </x:c>
+      <x:c r="D158" s="125" t="str">
+        <x:v>طلبات ترخيص الوكلاء</x:v>
+      </x:c>
+      <x:c r="E158" s="125" t="str">
+        <x:v>decide</x:v>
+      </x:c>
+      <x:c r="F158" s="125" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G158" s="125"/>
+      <x:c r="H158" s="125"/>
+      <x:c r="I158" s="125"/>
+      <x:c r="J158" s="125"/>
+      <x:c r="K158" s="125"/>
+      <x:c r="L158" s="125"/>
+      <x:c r="M158" s="125" t="str">
+        <x:v>قرار حسب الدور</x:v>
+      </x:c>
+      <x:c r="N158" s="125"/>
+      <x:c r="O158" s="125"/>
+      <x:c r="P158" s="125"/>
+      <x:c r="Q158" s="125"/>
+      <x:c r="R158" s="125"/>
+      <x:c r="S158" s="125"/>
+      <x:c r="T158" s="125" t="str">
+        <x:v>إضافة 2026-08-12: عام (كل الفروع) فقط. المنح تضبط من شاشة الأدوار؛ لا يوجد منح تلقائي أو create داخلي.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159">
+      <x:c r="A159" s="125" t="n">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="B159" s="125"/>
+      <x:c r="C159" s="125" t="str">
+        <x:v>agent_license.resolve_escalation</x:v>
+      </x:c>
+      <x:c r="D159" s="125" t="str">
+        <x:v>طلبات ترخيص الوكلاء</x:v>
+      </x:c>
+      <x:c r="E159" s="125" t="str">
+        <x:v>resolve_escalation</x:v>
+      </x:c>
+      <x:c r="F159" s="125" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G159" s="125"/>
+      <x:c r="H159" s="125"/>
+      <x:c r="I159" s="125"/>
+      <x:c r="J159" s="125"/>
+      <x:c r="K159" s="125"/>
+      <x:c r="L159" s="125"/>
+      <x:c r="M159" s="125" t="str">
+        <x:v>قرار حسب الدور</x:v>
+      </x:c>
+      <x:c r="N159" s="125"/>
+      <x:c r="O159" s="125"/>
+      <x:c r="P159" s="125"/>
+      <x:c r="Q159" s="125"/>
+      <x:c r="R159" s="125"/>
+      <x:c r="S159" s="125"/>
+      <x:c r="T159" s="125" t="str">
+        <x:v>إضافة 2026-08-12: عام (كل الفروع) فقط. المنح تضبط من شاشة الأدوار؛ لا يوجد منح تلقائي أو create داخلي.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160">
+      <x:c r="A160" s="125" t="n">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="B160" s="125"/>
+      <x:c r="C160" s="125" t="str">
+        <x:v>agent_license.archive</x:v>
+      </x:c>
+      <x:c r="D160" s="125" t="str">
+        <x:v>طلبات ترخيص الوكلاء</x:v>
+      </x:c>
+      <x:c r="E160" s="125" t="str">
+        <x:v>archive</x:v>
+      </x:c>
+      <x:c r="F160" s="125" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G160" s="125"/>
+      <x:c r="H160" s="125"/>
+      <x:c r="I160" s="125"/>
+      <x:c r="J160" s="125"/>
+      <x:c r="K160" s="125"/>
+      <x:c r="L160" s="125"/>
+      <x:c r="M160" s="125" t="str">
+        <x:v>قرار حسب الدور</x:v>
+      </x:c>
+      <x:c r="N160" s="125"/>
+      <x:c r="O160" s="125"/>
+      <x:c r="P160" s="125"/>
+      <x:c r="Q160" s="125"/>
+      <x:c r="R160" s="125"/>
+      <x:c r="S160" s="125"/>
+      <x:c r="T160" s="125" t="str">
+        <x:v>إضافة 2026-08-12: عام (كل الفروع) فقط. المنح تضبط من شاشة الأدوار؛ لا يوجد منح تلقائي أو create داخلي.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat(complaints): implement independent complaints domain
</commit_message>
<xml_diff>
--- a/صلاحيات_النظام.xlsx
+++ b/صلاحيات_النظام.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="كل الصلاحيات" sheetId="1" r:id="R9f522a626ff94e6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ملخص حسب الوحدة" sheetId="2" r:id="R1bcb52fa893243f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اختبار الأدوار" sheetId="3" r:id="R21312dd759e144c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اعتماد الزبائن" sheetId="4" r:id="R5e7f903561d842cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="كل الصلاحيات" sheetId="1" r:id="R33547e2c24ea4a03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ملخص حسب الوحدة" sheetId="2" r:id="Rd0650eeff7cf438c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اختبار الأدوار" sheetId="3" r:id="R9d7cc976be6a4692"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اعتماد الزبائن" sheetId="4" r:id="R5a4a35e6dddb4789"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -117,7 +117,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="43">
+  <x:fills count="44">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -329,6 +329,11 @@
         <x:fgColor rgb="FFC6EFCE"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC6EFCE"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -364,7 +369,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="128">
+  <x:cellXfs count="131">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -663,6 +668,9 @@
     <x:xf numFmtId="0" fontId="14" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="14" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -11031,6 +11039,1326 @@
         <x:v>إضافة 2026-08-16: استبدال روابط المنصات الخمس ذرياً مع التحقق والتدقيق؛ GLOBAL فقط، ولا يوجد منح تلقائي للأدوار.</x:v>
       </x:c>
     </x:row>
+    <x:row r="178">
+      <x:c r="A178" s="129" t="n">
+        <x:v>177</x:v>
+      </x:c>
+      <x:c r="B178" s="129"/>
+      <x:c r="C178" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D178" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E178" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="F178" s="129" t="str">
+        <x:v>view_list</x:v>
+      </x:c>
+      <x:c r="G178" s="129" t="str">
+        <x:v>عرض قائمة الشكاوى</x:v>
+      </x:c>
+      <x:c r="H178" s="129" t="str">
+        <x:v>complaints.view_list</x:v>
+      </x:c>
+      <x:c r="I178" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J178" s="129" t="n">
+        <x:v>310</x:v>
+      </x:c>
+      <x:c r="K178" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L178" s="129"/>
+      <x:c r="M178" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N178" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179">
+      <x:c r="A179" s="129" t="n">
+        <x:v>178</x:v>
+      </x:c>
+      <x:c r="B179" s="129"/>
+      <x:c r="C179" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D179" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E179" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="F179" s="129" t="str">
+        <x:v>view_details</x:v>
+      </x:c>
+      <x:c r="G179" s="129" t="str">
+        <x:v>عرض تفاصيل الشكوى</x:v>
+      </x:c>
+      <x:c r="H179" s="129" t="str">
+        <x:v>complaints.view_details</x:v>
+      </x:c>
+      <x:c r="I179" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J179" s="129" t="n">
+        <x:v>311</x:v>
+      </x:c>
+      <x:c r="K179" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L179" s="129"/>
+      <x:c r="M179" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N179" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180">
+      <x:c r="A180" s="129" t="n">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="B180" s="129"/>
+      <x:c r="C180" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D180" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E180" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="F180" s="129" t="str">
+        <x:v>create_internal</x:v>
+      </x:c>
+      <x:c r="G180" s="129" t="str">
+        <x:v>تسجيل شكوى من النظام</x:v>
+      </x:c>
+      <x:c r="H180" s="129" t="str">
+        <x:v>complaints.create_internal</x:v>
+      </x:c>
+      <x:c r="I180" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع</x:v>
+      </x:c>
+      <x:c r="J180" s="129" t="n">
+        <x:v>312</x:v>
+      </x:c>
+      <x:c r="K180" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L180" s="129"/>
+      <x:c r="M180" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N180" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181">
+      <x:c r="A181" s="129" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="B181" s="129"/>
+      <x:c r="C181" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D181" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E181" s="129" t="str">
+        <x:v>workflow</x:v>
+      </x:c>
+      <x:c r="F181" s="129" t="str">
+        <x:v>triage</x:v>
+      </x:c>
+      <x:c r="G181" s="129" t="str">
+        <x:v>فرز الشكاوى</x:v>
+      </x:c>
+      <x:c r="H181" s="129" t="str">
+        <x:v>complaints.triage</x:v>
+      </x:c>
+      <x:c r="I181" s="129" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J181" s="129" t="n">
+        <x:v>313</x:v>
+      </x:c>
+      <x:c r="K181" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L181" s="129"/>
+      <x:c r="M181" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N181" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182">
+      <x:c r="A182" s="129" t="n">
+        <x:v>181</x:v>
+      </x:c>
+      <x:c r="B182" s="129"/>
+      <x:c r="C182" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D182" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E182" s="129" t="str">
+        <x:v>workflow</x:v>
+      </x:c>
+      <x:c r="F182" s="129" t="str">
+        <x:v>change_type</x:v>
+      </x:c>
+      <x:c r="G182" s="129" t="str">
+        <x:v>تغيير نوع الشكوى</x:v>
+      </x:c>
+      <x:c r="H182" s="129" t="str">
+        <x:v>complaints.change_type</x:v>
+      </x:c>
+      <x:c r="I182" s="129" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J182" s="129" t="n">
+        <x:v>314</x:v>
+      </x:c>
+      <x:c r="K182" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L182" s="129"/>
+      <x:c r="M182" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N182" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183">
+      <x:c r="A183" s="129" t="n">
+        <x:v>182</x:v>
+      </x:c>
+      <x:c r="B183" s="129"/>
+      <x:c r="C183" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D183" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E183" s="129" t="str">
+        <x:v>workflow</x:v>
+      </x:c>
+      <x:c r="F183" s="129" t="str">
+        <x:v>change_priority</x:v>
+      </x:c>
+      <x:c r="G183" s="129" t="str">
+        <x:v>تغيير أولوية الشكوى</x:v>
+      </x:c>
+      <x:c r="H183" s="129" t="str">
+        <x:v>complaints.change_priority</x:v>
+      </x:c>
+      <x:c r="I183" s="129" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J183" s="129" t="n">
+        <x:v>315</x:v>
+      </x:c>
+      <x:c r="K183" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L183" s="129"/>
+      <x:c r="M183" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N183" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184">
+      <x:c r="A184" s="129" t="n">
+        <x:v>183</x:v>
+      </x:c>
+      <x:c r="B184" s="129"/>
+      <x:c r="C184" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D184" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E184" s="129" t="str">
+        <x:v>assignment</x:v>
+      </x:c>
+      <x:c r="F184" s="129" t="str">
+        <x:v>assign_branch</x:v>
+      </x:c>
+      <x:c r="G184" s="129" t="str">
+        <x:v>تعيين فرع معالجة</x:v>
+      </x:c>
+      <x:c r="H184" s="129" t="str">
+        <x:v>complaints.assign_branch</x:v>
+      </x:c>
+      <x:c r="I184" s="129" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J184" s="129" t="n">
+        <x:v>316</x:v>
+      </x:c>
+      <x:c r="K184" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L184" s="129"/>
+      <x:c r="M184" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N184" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185">
+      <x:c r="A185" s="129" t="n">
+        <x:v>184</x:v>
+      </x:c>
+      <x:c r="B185" s="129"/>
+      <x:c r="C185" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D185" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E185" s="129" t="str">
+        <x:v>assignment</x:v>
+      </x:c>
+      <x:c r="F185" s="129" t="str">
+        <x:v>transfer_branch</x:v>
+      </x:c>
+      <x:c r="G185" s="129" t="str">
+        <x:v>نقل فرع معالجة</x:v>
+      </x:c>
+      <x:c r="H185" s="129" t="str">
+        <x:v>complaints.transfer_branch</x:v>
+      </x:c>
+      <x:c r="I185" s="129" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J185" s="129" t="n">
+        <x:v>317</x:v>
+      </x:c>
+      <x:c r="K185" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L185" s="129"/>
+      <x:c r="M185" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N185" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186">
+      <x:c r="A186" s="129" t="n">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="B186" s="129"/>
+      <x:c r="C186" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D186" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E186" s="129" t="str">
+        <x:v>assignment</x:v>
+      </x:c>
+      <x:c r="F186" s="129" t="str">
+        <x:v>assign_handler</x:v>
+      </x:c>
+      <x:c r="G186" s="129" t="str">
+        <x:v>تعيين معالج شكوى</x:v>
+      </x:c>
+      <x:c r="H186" s="129" t="str">
+        <x:v>complaints.assign_handler</x:v>
+      </x:c>
+      <x:c r="I186" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع</x:v>
+      </x:c>
+      <x:c r="J186" s="129" t="n">
+        <x:v>318</x:v>
+      </x:c>
+      <x:c r="K186" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L186" s="129"/>
+      <x:c r="M186" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N186" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187">
+      <x:c r="A187" s="129" t="n">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="B187" s="129"/>
+      <x:c r="C187" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D187" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E187" s="129" t="str">
+        <x:v>assignment</x:v>
+      </x:c>
+      <x:c r="F187" s="129" t="str">
+        <x:v>reassign_handler</x:v>
+      </x:c>
+      <x:c r="G187" s="129" t="str">
+        <x:v>إعادة تعيين معالج شكوى</x:v>
+      </x:c>
+      <x:c r="H187" s="129" t="str">
+        <x:v>complaints.reassign_handler</x:v>
+      </x:c>
+      <x:c r="I187" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع</x:v>
+      </x:c>
+      <x:c r="J187" s="129" t="n">
+        <x:v>319</x:v>
+      </x:c>
+      <x:c r="K187" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L187" s="129"/>
+      <x:c r="M187" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N187" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188">
+      <x:c r="A188" s="129" t="n">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="B188" s="129"/>
+      <x:c r="C188" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D188" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E188" s="129" t="str">
+        <x:v>workflow</x:v>
+      </x:c>
+      <x:c r="F188" s="129" t="str">
+        <x:v>start_processing</x:v>
+      </x:c>
+      <x:c r="G188" s="129" t="str">
+        <x:v>بدء معالجة الشكوى</x:v>
+      </x:c>
+      <x:c r="H188" s="129" t="str">
+        <x:v>complaints.start_processing</x:v>
+      </x:c>
+      <x:c r="I188" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J188" s="129" t="n">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="K188" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L188" s="129"/>
+      <x:c r="M188" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N188" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189">
+      <x:c r="A189" s="129" t="n">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="B189" s="129"/>
+      <x:c r="C189" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D189" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E189" s="129" t="str">
+        <x:v>workflow</x:v>
+      </x:c>
+      <x:c r="F189" s="129" t="str">
+        <x:v>request_information</x:v>
+      </x:c>
+      <x:c r="G189" s="129" t="str">
+        <x:v>انتظار معلومات من مقدم الشكوى</x:v>
+      </x:c>
+      <x:c r="H189" s="129" t="str">
+        <x:v>complaints.request_information</x:v>
+      </x:c>
+      <x:c r="I189" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J189" s="129" t="n">
+        <x:v>321</x:v>
+      </x:c>
+      <x:c r="K189" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L189" s="129"/>
+      <x:c r="M189" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N189" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190">
+      <x:c r="A190" s="129" t="n">
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="B190" s="129"/>
+      <x:c r="C190" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D190" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E190" s="129" t="str">
+        <x:v>workflow</x:v>
+      </x:c>
+      <x:c r="F190" s="129" t="str">
+        <x:v>resume_processing</x:v>
+      </x:c>
+      <x:c r="G190" s="129" t="str">
+        <x:v>استئناف معالجة الشكوى</x:v>
+      </x:c>
+      <x:c r="H190" s="129" t="str">
+        <x:v>complaints.resume_processing</x:v>
+      </x:c>
+      <x:c r="I190" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J190" s="129" t="n">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="K190" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L190" s="129"/>
+      <x:c r="M190" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N190" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191">
+      <x:c r="A191" s="129" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="B191" s="129"/>
+      <x:c r="C191" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D191" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E191" s="129" t="str">
+        <x:v>workflow</x:v>
+      </x:c>
+      <x:c r="F191" s="129" t="str">
+        <x:v>resolve</x:v>
+      </x:c>
+      <x:c r="G191" s="129" t="str">
+        <x:v>حل الشكوى</x:v>
+      </x:c>
+      <x:c r="H191" s="129" t="str">
+        <x:v>complaints.resolve</x:v>
+      </x:c>
+      <x:c r="I191" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J191" s="129" t="n">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="K191" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L191" s="129"/>
+      <x:c r="M191" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N191" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192">
+      <x:c r="A192" s="129" t="n">
+        <x:v>191</x:v>
+      </x:c>
+      <x:c r="B192" s="129"/>
+      <x:c r="C192" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D192" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E192" s="129" t="str">
+        <x:v>workflow</x:v>
+      </x:c>
+      <x:c r="F192" s="129" t="str">
+        <x:v>close</x:v>
+      </x:c>
+      <x:c r="G192" s="129" t="str">
+        <x:v>إغلاق الشكوى</x:v>
+      </x:c>
+      <x:c r="H192" s="129" t="str">
+        <x:v>complaints.close</x:v>
+      </x:c>
+      <x:c r="I192" s="129" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J192" s="129" t="n">
+        <x:v>324</x:v>
+      </x:c>
+      <x:c r="K192" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L192" s="129"/>
+      <x:c r="M192" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N192" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193">
+      <x:c r="A193" s="129" t="n">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="B193" s="129"/>
+      <x:c r="C193" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D193" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E193" s="129" t="str">
+        <x:v>workflow</x:v>
+      </x:c>
+      <x:c r="F193" s="129" t="str">
+        <x:v>reject</x:v>
+      </x:c>
+      <x:c r="G193" s="129" t="str">
+        <x:v>رفض الشكوى</x:v>
+      </x:c>
+      <x:c r="H193" s="129" t="str">
+        <x:v>complaints.reject</x:v>
+      </x:c>
+      <x:c r="I193" s="129" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J193" s="129" t="n">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="K193" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L193" s="129"/>
+      <x:c r="M193" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N193" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194">
+      <x:c r="A194" s="129" t="n">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="B194" s="129"/>
+      <x:c r="C194" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D194" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E194" s="129" t="str">
+        <x:v>workflow</x:v>
+      </x:c>
+      <x:c r="F194" s="129" t="str">
+        <x:v>withdraw</x:v>
+      </x:c>
+      <x:c r="G194" s="129" t="str">
+        <x:v>تسجيل سحب الشكوى</x:v>
+      </x:c>
+      <x:c r="H194" s="129" t="str">
+        <x:v>complaints.withdraw</x:v>
+      </x:c>
+      <x:c r="I194" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J194" s="129" t="n">
+        <x:v>326</x:v>
+      </x:c>
+      <x:c r="K194" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L194" s="129"/>
+      <x:c r="M194" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N194" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195">
+      <x:c r="A195" s="129" t="n">
+        <x:v>194</x:v>
+      </x:c>
+      <x:c r="B195" s="129"/>
+      <x:c r="C195" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D195" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E195" s="129" t="str">
+        <x:v>workflow</x:v>
+      </x:c>
+      <x:c r="F195" s="129" t="str">
+        <x:v>reopen</x:v>
+      </x:c>
+      <x:c r="G195" s="129" t="str">
+        <x:v>إعادة فتح الشكوى</x:v>
+      </x:c>
+      <x:c r="H195" s="129" t="str">
+        <x:v>complaints.reopen</x:v>
+      </x:c>
+      <x:c r="I195" s="129" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J195" s="129" t="n">
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="K195" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L195" s="129"/>
+      <x:c r="M195" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N195" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196">
+      <x:c r="A196" s="129" t="n">
+        <x:v>195</x:v>
+      </x:c>
+      <x:c r="B196" s="129"/>
+      <x:c r="C196" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D196" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E196" s="129" t="str">
+        <x:v>workflow</x:v>
+      </x:c>
+      <x:c r="F196" s="129" t="str">
+        <x:v>review_duplicates</x:v>
+      </x:c>
+      <x:c r="G196" s="129" t="str">
+        <x:v>مراجعة تكرار الشكاوى</x:v>
+      </x:c>
+      <x:c r="H196" s="129" t="str">
+        <x:v>complaints.review_duplicates</x:v>
+      </x:c>
+      <x:c r="I196" s="129" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J196" s="129" t="n">
+        <x:v>328</x:v>
+      </x:c>
+      <x:c r="K196" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L196" s="129"/>
+      <x:c r="M196" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N196" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197">
+      <x:c r="A197" s="129" t="n">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="B197" s="129"/>
+      <x:c r="C197" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D197" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E197" s="129" t="str">
+        <x:v>notes</x:v>
+      </x:c>
+      <x:c r="F197" s="129" t="str">
+        <x:v>add_internal_note</x:v>
+      </x:c>
+      <x:c r="G197" s="129" t="str">
+        <x:v>إضافة ملاحظة داخلية</x:v>
+      </x:c>
+      <x:c r="H197" s="129" t="str">
+        <x:v>complaints.add_internal_note</x:v>
+      </x:c>
+      <x:c r="I197" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J197" s="129" t="n">
+        <x:v>329</x:v>
+      </x:c>
+      <x:c r="K197" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L197" s="129"/>
+      <x:c r="M197" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N197" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="198">
+      <x:c r="A198" s="129" t="n">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="B198" s="129"/>
+      <x:c r="C198" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D198" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E198" s="129" t="str">
+        <x:v>updates</x:v>
+      </x:c>
+      <x:c r="F198" s="129" t="str">
+        <x:v>publish_update</x:v>
+      </x:c>
+      <x:c r="G198" s="129" t="str">
+        <x:v>نشر تحديث لمقدم الشكوى</x:v>
+      </x:c>
+      <x:c r="H198" s="129" t="str">
+        <x:v>complaints.publish_update</x:v>
+      </x:c>
+      <x:c r="I198" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J198" s="129" t="n">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="K198" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L198" s="129"/>
+      <x:c r="M198" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N198" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199">
+      <x:c r="A199" s="129" t="n">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="B199" s="129"/>
+      <x:c r="C199" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D199" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E199" s="129" t="str">
+        <x:v>attachments</x:v>
+      </x:c>
+      <x:c r="F199" s="129" t="str">
+        <x:v>view</x:v>
+      </x:c>
+      <x:c r="G199" s="129" t="str">
+        <x:v>عرض صور الشكوى</x:v>
+      </x:c>
+      <x:c r="H199" s="129" t="str">
+        <x:v>complaints.view_attachments</x:v>
+      </x:c>
+      <x:c r="I199" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J199" s="129" t="n">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="K199" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L199" s="129"/>
+      <x:c r="M199" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N199" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200">
+      <x:c r="A200" s="129" t="n">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="B200" s="129"/>
+      <x:c r="C200" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D200" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E200" s="129" t="str">
+        <x:v>attachments</x:v>
+      </x:c>
+      <x:c r="F200" s="129" t="str">
+        <x:v>download</x:v>
+      </x:c>
+      <x:c r="G200" s="129" t="str">
+        <x:v>تنزيل صور الشكوى</x:v>
+      </x:c>
+      <x:c r="H200" s="129" t="str">
+        <x:v>complaints.download_attachments</x:v>
+      </x:c>
+      <x:c r="I200" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J200" s="129" t="n">
+        <x:v>332</x:v>
+      </x:c>
+      <x:c r="K200" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L200" s="129"/>
+      <x:c r="M200" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N200" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201">
+      <x:c r="A201" s="129" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="B201" s="129"/>
+      <x:c r="C201" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D201" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E201" s="129" t="str">
+        <x:v>audit</x:v>
+      </x:c>
+      <x:c r="F201" s="129" t="str">
+        <x:v>view</x:v>
+      </x:c>
+      <x:c r="G201" s="129" t="str">
+        <x:v>عرض سجل تدقيق الشكوى</x:v>
+      </x:c>
+      <x:c r="H201" s="129" t="str">
+        <x:v>complaints.view_audit</x:v>
+      </x:c>
+      <x:c r="I201" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J201" s="129" t="n">
+        <x:v>333</x:v>
+      </x:c>
+      <x:c r="K201" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L201" s="129"/>
+      <x:c r="M201" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N201" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202">
+      <x:c r="A202" s="129" t="n">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="B202" s="129"/>
+      <x:c r="C202" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D202" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E202" s="129" t="str">
+        <x:v>reports</x:v>
+      </x:c>
+      <x:c r="F202" s="129" t="str">
+        <x:v>view</x:v>
+      </x:c>
+      <x:c r="G202" s="129" t="str">
+        <x:v>عرض تقارير الشكاوى</x:v>
+      </x:c>
+      <x:c r="H202" s="129" t="str">
+        <x:v>complaints.view_reports</x:v>
+      </x:c>
+      <x:c r="I202" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع</x:v>
+      </x:c>
+      <x:c r="J202" s="129" t="n">
+        <x:v>334</x:v>
+      </x:c>
+      <x:c r="K202" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L202" s="129"/>
+      <x:c r="M202" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N202" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203">
+      <x:c r="A203" s="129" t="n">
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="B203" s="129"/>
+      <x:c r="C203" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D203" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E203" s="129" t="str">
+        <x:v>reports</x:v>
+      </x:c>
+      <x:c r="F203" s="129" t="str">
+        <x:v>export</x:v>
+      </x:c>
+      <x:c r="G203" s="129" t="str">
+        <x:v>تصدير الشكاوى</x:v>
+      </x:c>
+      <x:c r="H203" s="129" t="str">
+        <x:v>complaints.export</x:v>
+      </x:c>
+      <x:c r="I203" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع</x:v>
+      </x:c>
+      <x:c r="J203" s="129" t="n">
+        <x:v>335</x:v>
+      </x:c>
+      <x:c r="K203" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L203" s="129"/>
+      <x:c r="M203" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N203" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204">
+      <x:c r="A204" s="129" t="n">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="B204" s="129"/>
+      <x:c r="C204" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D204" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E204" s="129" t="str">
+        <x:v>links</x:v>
+      </x:c>
+      <x:c r="F204" s="129" t="str">
+        <x:v>link_requester</x:v>
+      </x:c>
+      <x:c r="G204" s="129" t="str">
+        <x:v>ربط مقدم الشكوى</x:v>
+      </x:c>
+      <x:c r="H204" s="129" t="str">
+        <x:v>complaints.link_requester</x:v>
+      </x:c>
+      <x:c r="I204" s="129" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J204" s="129" t="n">
+        <x:v>336</x:v>
+      </x:c>
+      <x:c r="K204" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L204" s="129"/>
+      <x:c r="M204" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N204" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205">
+      <x:c r="A205" s="129" t="n">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="B205" s="129"/>
+      <x:c r="C205" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D205" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E205" s="129" t="str">
+        <x:v>links</x:v>
+      </x:c>
+      <x:c r="F205" s="129" t="str">
+        <x:v>link_visit</x:v>
+      </x:c>
+      <x:c r="G205" s="129" t="str">
+        <x:v>ربط زيارة بالشكوى</x:v>
+      </x:c>
+      <x:c r="H205" s="129" t="str">
+        <x:v>complaints.link_visit</x:v>
+      </x:c>
+      <x:c r="I205" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J205" s="129" t="n">
+        <x:v>337</x:v>
+      </x:c>
+      <x:c r="K205" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L205" s="129"/>
+      <x:c r="M205" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N205" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206">
+      <x:c r="A206" s="129" t="n">
+        <x:v>205</x:v>
+      </x:c>
+      <x:c r="B206" s="129"/>
+      <x:c r="C206" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D206" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E206" s="129" t="str">
+        <x:v>links</x:v>
+      </x:c>
+      <x:c r="F206" s="129" t="str">
+        <x:v>link_device</x:v>
+      </x:c>
+      <x:c r="G206" s="129" t="str">
+        <x:v>ربط جهاز بالشكوى</x:v>
+      </x:c>
+      <x:c r="H206" s="129" t="str">
+        <x:v>complaints.link_device</x:v>
+      </x:c>
+      <x:c r="I206" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J206" s="129" t="n">
+        <x:v>338</x:v>
+      </x:c>
+      <x:c r="K206" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L206" s="129"/>
+      <x:c r="M206" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N206" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="207">
+      <x:c r="A207" s="129" t="n">
+        <x:v>206</x:v>
+      </x:c>
+      <x:c r="B207" s="129"/>
+      <x:c r="C207" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D207" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E207" s="129" t="str">
+        <x:v>links</x:v>
+      </x:c>
+      <x:c r="F207" s="129" t="str">
+        <x:v>link_target</x:v>
+      </x:c>
+      <x:c r="G207" s="129" t="str">
+        <x:v>ربط الجهة المشكو عليها</x:v>
+      </x:c>
+      <x:c r="H207" s="129" t="str">
+        <x:v>complaints.link_target</x:v>
+      </x:c>
+      <x:c r="I207" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J207" s="129" t="n">
+        <x:v>339</x:v>
+      </x:c>
+      <x:c r="K207" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L207" s="129"/>
+      <x:c r="M207" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N207" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="208">
+      <x:c r="A208" s="129" t="n">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="B208" s="129"/>
+      <x:c r="C208" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D208" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E208" s="129" t="str">
+        <x:v>links</x:v>
+      </x:c>
+      <x:c r="F208" s="129" t="str">
+        <x:v>link_work</x:v>
+      </x:c>
+      <x:c r="G208" s="129" t="str">
+        <x:v>ربط عمل تشغيلي بالشكوى</x:v>
+      </x:c>
+      <x:c r="H208" s="129" t="str">
+        <x:v>complaints.link_operational_work</x:v>
+      </x:c>
+      <x:c r="I208" s="129" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J208" s="129" t="n">
+        <x:v>340</x:v>
+      </x:c>
+      <x:c r="K208" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L208" s="129"/>
+      <x:c r="M208" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N208" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209">
+      <x:c r="A209" s="129" t="n">
+        <x:v>208</x:v>
+      </x:c>
+      <x:c r="B209" s="129"/>
+      <x:c r="C209" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D209" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E209" s="129" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="F209" s="129" t="str">
+        <x:v>duplicates</x:v>
+      </x:c>
+      <x:c r="G209" s="129" t="str">
+        <x:v>إدارة إعدادات تكرار الشكاوى</x:v>
+      </x:c>
+      <x:c r="H209" s="129" t="str">
+        <x:v>complaints.manage_duplicate_settings</x:v>
+      </x:c>
+      <x:c r="I209" s="129" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J209" s="129" t="n">
+        <x:v>341</x:v>
+      </x:c>
+      <x:c r="K209" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L209" s="129"/>
+      <x:c r="M209" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N209" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="210">
+      <x:c r="A210" s="129" t="n">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="B210" s="129"/>
+      <x:c r="C210" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="D210" s="129" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="E210" s="129" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="F210" s="129" t="str">
+        <x:v>abuse</x:v>
+      </x:c>
+      <x:c r="G210" s="129" t="str">
+        <x:v>إدارة حدود تقديم الشكاوى</x:v>
+      </x:c>
+      <x:c r="H210" s="129" t="str">
+        <x:v>complaints.manage_abuse_settings</x:v>
+      </x:c>
+      <x:c r="I210" s="129" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J210" s="129" t="n">
+        <x:v>342</x:v>
+      </x:c>
+      <x:c r="K210" s="129" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L210" s="129"/>
+      <x:c r="M210" s="129" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N210" s="129" t="str">
+        <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11433,12 +12761,23 @@
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" t="str">
+      <x:c r="A28" s="130" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="B28" s="130" t="str">
+        <x:v>complaints</x:v>
+      </x:c>
+      <x:c r="C28" s="130" t="n">
+        <x:v>33</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
         <x:v>الإجمالي</x:v>
       </x:c>
-      <x:c r="B28"/>
-      <x:c r="C28" t="n">
-        <x:v>176</x:v>
+      <x:c r="B29"/>
+      <x:c r="C29" t="n">
+        <x:v>209</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -19018,6 +20357,1194 @@
         <x:v>إضافة 2026-08-16: استبدال روابط المنصات الخمس ذرياً مع التحقق والتدقيق؛ GLOBAL فقط، ولا يوجد منح تلقائي للأدوار.</x:v>
       </x:c>
     </x:row>
+    <x:row r="165">
+      <x:c r="A165" s="129" t="n">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="B165" s="129"/>
+      <x:c r="C165" s="129" t="str">
+        <x:v>complaints.view_list</x:v>
+      </x:c>
+      <x:c r="D165" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E165" s="129" t="str">
+        <x:v>view_list</x:v>
+      </x:c>
+      <x:c r="F165" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G165" s="129"/>
+      <x:c r="H165" s="129"/>
+      <x:c r="I165" s="129"/>
+      <x:c r="J165" s="129"/>
+      <x:c r="K165" s="129"/>
+      <x:c r="L165" s="129"/>
+      <x:c r="M165" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N165" s="129"/>
+      <x:c r="O165" s="129"/>
+      <x:c r="P165" s="129"/>
+      <x:c r="Q165" s="129"/>
+      <x:c r="R165" s="129"/>
+      <x:c r="S165" s="129"/>
+      <x:c r="T165" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH / ASSIGNED. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166">
+      <x:c r="A166" s="129" t="n">
+        <x:v>165</x:v>
+      </x:c>
+      <x:c r="B166" s="129"/>
+      <x:c r="C166" s="129" t="str">
+        <x:v>complaints.view_details</x:v>
+      </x:c>
+      <x:c r="D166" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E166" s="129" t="str">
+        <x:v>view_details</x:v>
+      </x:c>
+      <x:c r="F166" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G166" s="129"/>
+      <x:c r="H166" s="129"/>
+      <x:c r="I166" s="129"/>
+      <x:c r="J166" s="129"/>
+      <x:c r="K166" s="129"/>
+      <x:c r="L166" s="129"/>
+      <x:c r="M166" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N166" s="129"/>
+      <x:c r="O166" s="129"/>
+      <x:c r="P166" s="129"/>
+      <x:c r="Q166" s="129"/>
+      <x:c r="R166" s="129"/>
+      <x:c r="S166" s="129"/>
+      <x:c r="T166" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH / ASSIGNED. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167">
+      <x:c r="A167" s="129" t="n">
+        <x:v>166</x:v>
+      </x:c>
+      <x:c r="B167" s="129"/>
+      <x:c r="C167" s="129" t="str">
+        <x:v>complaints.create_internal</x:v>
+      </x:c>
+      <x:c r="D167" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E167" s="129" t="str">
+        <x:v>create_internal</x:v>
+      </x:c>
+      <x:c r="F167" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G167" s="129"/>
+      <x:c r="H167" s="129"/>
+      <x:c r="I167" s="129"/>
+      <x:c r="J167" s="129"/>
+      <x:c r="K167" s="129"/>
+      <x:c r="L167" s="129"/>
+      <x:c r="M167" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N167" s="129"/>
+      <x:c r="O167" s="129"/>
+      <x:c r="P167" s="129"/>
+      <x:c r="Q167" s="129"/>
+      <x:c r="R167" s="129"/>
+      <x:c r="S167" s="129"/>
+      <x:c r="T167" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168">
+      <x:c r="A168" s="129" t="n">
+        <x:v>167</x:v>
+      </x:c>
+      <x:c r="B168" s="129"/>
+      <x:c r="C168" s="129" t="str">
+        <x:v>complaints.triage</x:v>
+      </x:c>
+      <x:c r="D168" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E168" s="129" t="str">
+        <x:v>triage</x:v>
+      </x:c>
+      <x:c r="F168" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G168" s="129"/>
+      <x:c r="H168" s="129"/>
+      <x:c r="I168" s="129"/>
+      <x:c r="J168" s="129"/>
+      <x:c r="K168" s="129"/>
+      <x:c r="L168" s="129"/>
+      <x:c r="M168" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N168" s="129"/>
+      <x:c r="O168" s="129"/>
+      <x:c r="P168" s="129"/>
+      <x:c r="Q168" s="129"/>
+      <x:c r="R168" s="129"/>
+      <x:c r="S168" s="129"/>
+      <x:c r="T168" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169">
+      <x:c r="A169" s="129" t="n">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="B169" s="129"/>
+      <x:c r="C169" s="129" t="str">
+        <x:v>complaints.change_type</x:v>
+      </x:c>
+      <x:c r="D169" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E169" s="129" t="str">
+        <x:v>change_type</x:v>
+      </x:c>
+      <x:c r="F169" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G169" s="129"/>
+      <x:c r="H169" s="129"/>
+      <x:c r="I169" s="129"/>
+      <x:c r="J169" s="129"/>
+      <x:c r="K169" s="129"/>
+      <x:c r="L169" s="129"/>
+      <x:c r="M169" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N169" s="129"/>
+      <x:c r="O169" s="129"/>
+      <x:c r="P169" s="129"/>
+      <x:c r="Q169" s="129"/>
+      <x:c r="R169" s="129"/>
+      <x:c r="S169" s="129"/>
+      <x:c r="T169" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170">
+      <x:c r="A170" s="129" t="n">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="B170" s="129"/>
+      <x:c r="C170" s="129" t="str">
+        <x:v>complaints.change_priority</x:v>
+      </x:c>
+      <x:c r="D170" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E170" s="129" t="str">
+        <x:v>change_priority</x:v>
+      </x:c>
+      <x:c r="F170" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G170" s="129"/>
+      <x:c r="H170" s="129"/>
+      <x:c r="I170" s="129"/>
+      <x:c r="J170" s="129"/>
+      <x:c r="K170" s="129"/>
+      <x:c r="L170" s="129"/>
+      <x:c r="M170" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N170" s="129"/>
+      <x:c r="O170" s="129"/>
+      <x:c r="P170" s="129"/>
+      <x:c r="Q170" s="129"/>
+      <x:c r="R170" s="129"/>
+      <x:c r="S170" s="129"/>
+      <x:c r="T170" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171">
+      <x:c r="A171" s="129" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="B171" s="129"/>
+      <x:c r="C171" s="129" t="str">
+        <x:v>complaints.assign_branch</x:v>
+      </x:c>
+      <x:c r="D171" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E171" s="129" t="str">
+        <x:v>assign_branch</x:v>
+      </x:c>
+      <x:c r="F171" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G171" s="129"/>
+      <x:c r="H171" s="129"/>
+      <x:c r="I171" s="129"/>
+      <x:c r="J171" s="129"/>
+      <x:c r="K171" s="129"/>
+      <x:c r="L171" s="129"/>
+      <x:c r="M171" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N171" s="129"/>
+      <x:c r="O171" s="129"/>
+      <x:c r="P171" s="129"/>
+      <x:c r="Q171" s="129"/>
+      <x:c r="R171" s="129"/>
+      <x:c r="S171" s="129"/>
+      <x:c r="T171" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" s="129" t="n">
+        <x:v>171</x:v>
+      </x:c>
+      <x:c r="B172" s="129"/>
+      <x:c r="C172" s="129" t="str">
+        <x:v>complaints.transfer_branch</x:v>
+      </x:c>
+      <x:c r="D172" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E172" s="129" t="str">
+        <x:v>transfer_branch</x:v>
+      </x:c>
+      <x:c r="F172" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G172" s="129"/>
+      <x:c r="H172" s="129"/>
+      <x:c r="I172" s="129"/>
+      <x:c r="J172" s="129"/>
+      <x:c r="K172" s="129"/>
+      <x:c r="L172" s="129"/>
+      <x:c r="M172" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N172" s="129"/>
+      <x:c r="O172" s="129"/>
+      <x:c r="P172" s="129"/>
+      <x:c r="Q172" s="129"/>
+      <x:c r="R172" s="129"/>
+      <x:c r="S172" s="129"/>
+      <x:c r="T172" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173">
+      <x:c r="A173" s="129" t="n">
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="B173" s="129"/>
+      <x:c r="C173" s="129" t="str">
+        <x:v>complaints.assign_handler</x:v>
+      </x:c>
+      <x:c r="D173" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E173" s="129" t="str">
+        <x:v>assign_handler</x:v>
+      </x:c>
+      <x:c r="F173" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G173" s="129"/>
+      <x:c r="H173" s="129"/>
+      <x:c r="I173" s="129"/>
+      <x:c r="J173" s="129"/>
+      <x:c r="K173" s="129"/>
+      <x:c r="L173" s="129"/>
+      <x:c r="M173" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N173" s="129"/>
+      <x:c r="O173" s="129"/>
+      <x:c r="P173" s="129"/>
+      <x:c r="Q173" s="129"/>
+      <x:c r="R173" s="129"/>
+      <x:c r="S173" s="129"/>
+      <x:c r="T173" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174">
+      <x:c r="A174" s="129" t="n">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="B174" s="129"/>
+      <x:c r="C174" s="129" t="str">
+        <x:v>complaints.reassign_handler</x:v>
+      </x:c>
+      <x:c r="D174" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E174" s="129" t="str">
+        <x:v>reassign_handler</x:v>
+      </x:c>
+      <x:c r="F174" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G174" s="129"/>
+      <x:c r="H174" s="129"/>
+      <x:c r="I174" s="129"/>
+      <x:c r="J174" s="129"/>
+      <x:c r="K174" s="129"/>
+      <x:c r="L174" s="129"/>
+      <x:c r="M174" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N174" s="129"/>
+      <x:c r="O174" s="129"/>
+      <x:c r="P174" s="129"/>
+      <x:c r="Q174" s="129"/>
+      <x:c r="R174" s="129"/>
+      <x:c r="S174" s="129"/>
+      <x:c r="T174" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175">
+      <x:c r="A175" s="129" t="n">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="B175" s="129"/>
+      <x:c r="C175" s="129" t="str">
+        <x:v>complaints.start_processing</x:v>
+      </x:c>
+      <x:c r="D175" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E175" s="129" t="str">
+        <x:v>start_processing</x:v>
+      </x:c>
+      <x:c r="F175" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G175" s="129"/>
+      <x:c r="H175" s="129"/>
+      <x:c r="I175" s="129"/>
+      <x:c r="J175" s="129"/>
+      <x:c r="K175" s="129"/>
+      <x:c r="L175" s="129"/>
+      <x:c r="M175" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N175" s="129"/>
+      <x:c r="O175" s="129"/>
+      <x:c r="P175" s="129"/>
+      <x:c r="Q175" s="129"/>
+      <x:c r="R175" s="129"/>
+      <x:c r="S175" s="129"/>
+      <x:c r="T175" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH / ASSIGNED. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176">
+      <x:c r="A176" s="129" t="n">
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="B176" s="129"/>
+      <x:c r="C176" s="129" t="str">
+        <x:v>complaints.request_information</x:v>
+      </x:c>
+      <x:c r="D176" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E176" s="129" t="str">
+        <x:v>request_information</x:v>
+      </x:c>
+      <x:c r="F176" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G176" s="129"/>
+      <x:c r="H176" s="129"/>
+      <x:c r="I176" s="129"/>
+      <x:c r="J176" s="129"/>
+      <x:c r="K176" s="129"/>
+      <x:c r="L176" s="129"/>
+      <x:c r="M176" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N176" s="129"/>
+      <x:c r="O176" s="129"/>
+      <x:c r="P176" s="129"/>
+      <x:c r="Q176" s="129"/>
+      <x:c r="R176" s="129"/>
+      <x:c r="S176" s="129"/>
+      <x:c r="T176" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH / ASSIGNED. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177">
+      <x:c r="A177" s="129" t="n">
+        <x:v>176</x:v>
+      </x:c>
+      <x:c r="B177" s="129"/>
+      <x:c r="C177" s="129" t="str">
+        <x:v>complaints.resume_processing</x:v>
+      </x:c>
+      <x:c r="D177" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E177" s="129" t="str">
+        <x:v>resume_processing</x:v>
+      </x:c>
+      <x:c r="F177" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G177" s="129"/>
+      <x:c r="H177" s="129"/>
+      <x:c r="I177" s="129"/>
+      <x:c r="J177" s="129"/>
+      <x:c r="K177" s="129"/>
+      <x:c r="L177" s="129"/>
+      <x:c r="M177" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N177" s="129"/>
+      <x:c r="O177" s="129"/>
+      <x:c r="P177" s="129"/>
+      <x:c r="Q177" s="129"/>
+      <x:c r="R177" s="129"/>
+      <x:c r="S177" s="129"/>
+      <x:c r="T177" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH / ASSIGNED. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178">
+      <x:c r="A178" s="129" t="n">
+        <x:v>177</x:v>
+      </x:c>
+      <x:c r="B178" s="129"/>
+      <x:c r="C178" s="129" t="str">
+        <x:v>complaints.resolve</x:v>
+      </x:c>
+      <x:c r="D178" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E178" s="129" t="str">
+        <x:v>resolve</x:v>
+      </x:c>
+      <x:c r="F178" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G178" s="129"/>
+      <x:c r="H178" s="129"/>
+      <x:c r="I178" s="129"/>
+      <x:c r="J178" s="129"/>
+      <x:c r="K178" s="129"/>
+      <x:c r="L178" s="129"/>
+      <x:c r="M178" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N178" s="129"/>
+      <x:c r="O178" s="129"/>
+      <x:c r="P178" s="129"/>
+      <x:c r="Q178" s="129"/>
+      <x:c r="R178" s="129"/>
+      <x:c r="S178" s="129"/>
+      <x:c r="T178" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH / ASSIGNED. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179">
+      <x:c r="A179" s="129" t="n">
+        <x:v>178</x:v>
+      </x:c>
+      <x:c r="B179" s="129"/>
+      <x:c r="C179" s="129" t="str">
+        <x:v>complaints.close</x:v>
+      </x:c>
+      <x:c r="D179" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E179" s="129" t="str">
+        <x:v>close</x:v>
+      </x:c>
+      <x:c r="F179" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G179" s="129"/>
+      <x:c r="H179" s="129"/>
+      <x:c r="I179" s="129"/>
+      <x:c r="J179" s="129"/>
+      <x:c r="K179" s="129"/>
+      <x:c r="L179" s="129"/>
+      <x:c r="M179" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N179" s="129"/>
+      <x:c r="O179" s="129"/>
+      <x:c r="P179" s="129"/>
+      <x:c r="Q179" s="129"/>
+      <x:c r="R179" s="129"/>
+      <x:c r="S179" s="129"/>
+      <x:c r="T179" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180">
+      <x:c r="A180" s="129" t="n">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="B180" s="129"/>
+      <x:c r="C180" s="129" t="str">
+        <x:v>complaints.reject</x:v>
+      </x:c>
+      <x:c r="D180" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E180" s="129" t="str">
+        <x:v>reject</x:v>
+      </x:c>
+      <x:c r="F180" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G180" s="129"/>
+      <x:c r="H180" s="129"/>
+      <x:c r="I180" s="129"/>
+      <x:c r="J180" s="129"/>
+      <x:c r="K180" s="129"/>
+      <x:c r="L180" s="129"/>
+      <x:c r="M180" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N180" s="129"/>
+      <x:c r="O180" s="129"/>
+      <x:c r="P180" s="129"/>
+      <x:c r="Q180" s="129"/>
+      <x:c r="R180" s="129"/>
+      <x:c r="S180" s="129"/>
+      <x:c r="T180" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181">
+      <x:c r="A181" s="129" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="B181" s="129"/>
+      <x:c r="C181" s="129" t="str">
+        <x:v>complaints.withdraw</x:v>
+      </x:c>
+      <x:c r="D181" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E181" s="129" t="str">
+        <x:v>withdraw</x:v>
+      </x:c>
+      <x:c r="F181" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G181" s="129"/>
+      <x:c r="H181" s="129"/>
+      <x:c r="I181" s="129"/>
+      <x:c r="J181" s="129"/>
+      <x:c r="K181" s="129"/>
+      <x:c r="L181" s="129"/>
+      <x:c r="M181" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N181" s="129"/>
+      <x:c r="O181" s="129"/>
+      <x:c r="P181" s="129"/>
+      <x:c r="Q181" s="129"/>
+      <x:c r="R181" s="129"/>
+      <x:c r="S181" s="129"/>
+      <x:c r="T181" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH / ASSIGNED. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182">
+      <x:c r="A182" s="129" t="n">
+        <x:v>181</x:v>
+      </x:c>
+      <x:c r="B182" s="129"/>
+      <x:c r="C182" s="129" t="str">
+        <x:v>complaints.reopen</x:v>
+      </x:c>
+      <x:c r="D182" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E182" s="129" t="str">
+        <x:v>reopen</x:v>
+      </x:c>
+      <x:c r="F182" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G182" s="129"/>
+      <x:c r="H182" s="129"/>
+      <x:c r="I182" s="129"/>
+      <x:c r="J182" s="129"/>
+      <x:c r="K182" s="129"/>
+      <x:c r="L182" s="129"/>
+      <x:c r="M182" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N182" s="129"/>
+      <x:c r="O182" s="129"/>
+      <x:c r="P182" s="129"/>
+      <x:c r="Q182" s="129"/>
+      <x:c r="R182" s="129"/>
+      <x:c r="S182" s="129"/>
+      <x:c r="T182" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183">
+      <x:c r="A183" s="129" t="n">
+        <x:v>182</x:v>
+      </x:c>
+      <x:c r="B183" s="129"/>
+      <x:c r="C183" s="129" t="str">
+        <x:v>complaints.review_duplicates</x:v>
+      </x:c>
+      <x:c r="D183" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E183" s="129" t="str">
+        <x:v>review_duplicates</x:v>
+      </x:c>
+      <x:c r="F183" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G183" s="129"/>
+      <x:c r="H183" s="129"/>
+      <x:c r="I183" s="129"/>
+      <x:c r="J183" s="129"/>
+      <x:c r="K183" s="129"/>
+      <x:c r="L183" s="129"/>
+      <x:c r="M183" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N183" s="129"/>
+      <x:c r="O183" s="129"/>
+      <x:c r="P183" s="129"/>
+      <x:c r="Q183" s="129"/>
+      <x:c r="R183" s="129"/>
+      <x:c r="S183" s="129"/>
+      <x:c r="T183" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184">
+      <x:c r="A184" s="129" t="n">
+        <x:v>183</x:v>
+      </x:c>
+      <x:c r="B184" s="129"/>
+      <x:c r="C184" s="129" t="str">
+        <x:v>complaints.add_internal_note</x:v>
+      </x:c>
+      <x:c r="D184" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E184" s="129" t="str">
+        <x:v>add_internal_note</x:v>
+      </x:c>
+      <x:c r="F184" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G184" s="129"/>
+      <x:c r="H184" s="129"/>
+      <x:c r="I184" s="129"/>
+      <x:c r="J184" s="129"/>
+      <x:c r="K184" s="129"/>
+      <x:c r="L184" s="129"/>
+      <x:c r="M184" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N184" s="129"/>
+      <x:c r="O184" s="129"/>
+      <x:c r="P184" s="129"/>
+      <x:c r="Q184" s="129"/>
+      <x:c r="R184" s="129"/>
+      <x:c r="S184" s="129"/>
+      <x:c r="T184" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH / ASSIGNED. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185">
+      <x:c r="A185" s="129" t="n">
+        <x:v>184</x:v>
+      </x:c>
+      <x:c r="B185" s="129"/>
+      <x:c r="C185" s="129" t="str">
+        <x:v>complaints.publish_update</x:v>
+      </x:c>
+      <x:c r="D185" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E185" s="129" t="str">
+        <x:v>publish_update</x:v>
+      </x:c>
+      <x:c r="F185" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G185" s="129"/>
+      <x:c r="H185" s="129"/>
+      <x:c r="I185" s="129"/>
+      <x:c r="J185" s="129"/>
+      <x:c r="K185" s="129"/>
+      <x:c r="L185" s="129"/>
+      <x:c r="M185" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N185" s="129"/>
+      <x:c r="O185" s="129"/>
+      <x:c r="P185" s="129"/>
+      <x:c r="Q185" s="129"/>
+      <x:c r="R185" s="129"/>
+      <x:c r="S185" s="129"/>
+      <x:c r="T185" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH / ASSIGNED. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186">
+      <x:c r="A186" s="129" t="n">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="B186" s="129"/>
+      <x:c r="C186" s="129" t="str">
+        <x:v>complaints.view_attachments</x:v>
+      </x:c>
+      <x:c r="D186" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E186" s="129" t="str">
+        <x:v>view</x:v>
+      </x:c>
+      <x:c r="F186" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G186" s="129"/>
+      <x:c r="H186" s="129"/>
+      <x:c r="I186" s="129"/>
+      <x:c r="J186" s="129"/>
+      <x:c r="K186" s="129"/>
+      <x:c r="L186" s="129"/>
+      <x:c r="M186" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N186" s="129"/>
+      <x:c r="O186" s="129"/>
+      <x:c r="P186" s="129"/>
+      <x:c r="Q186" s="129"/>
+      <x:c r="R186" s="129"/>
+      <x:c r="S186" s="129"/>
+      <x:c r="T186" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH / ASSIGNED. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187">
+      <x:c r="A187" s="129" t="n">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="B187" s="129"/>
+      <x:c r="C187" s="129" t="str">
+        <x:v>complaints.download_attachments</x:v>
+      </x:c>
+      <x:c r="D187" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E187" s="129" t="str">
+        <x:v>download</x:v>
+      </x:c>
+      <x:c r="F187" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G187" s="129"/>
+      <x:c r="H187" s="129"/>
+      <x:c r="I187" s="129"/>
+      <x:c r="J187" s="129"/>
+      <x:c r="K187" s="129"/>
+      <x:c r="L187" s="129"/>
+      <x:c r="M187" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N187" s="129"/>
+      <x:c r="O187" s="129"/>
+      <x:c r="P187" s="129"/>
+      <x:c r="Q187" s="129"/>
+      <x:c r="R187" s="129"/>
+      <x:c r="S187" s="129"/>
+      <x:c r="T187" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH / ASSIGNED. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188">
+      <x:c r="A188" s="129" t="n">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="B188" s="129"/>
+      <x:c r="C188" s="129" t="str">
+        <x:v>complaints.view_audit</x:v>
+      </x:c>
+      <x:c r="D188" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E188" s="129" t="str">
+        <x:v>view</x:v>
+      </x:c>
+      <x:c r="F188" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G188" s="129"/>
+      <x:c r="H188" s="129"/>
+      <x:c r="I188" s="129"/>
+      <x:c r="J188" s="129"/>
+      <x:c r="K188" s="129"/>
+      <x:c r="L188" s="129"/>
+      <x:c r="M188" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N188" s="129"/>
+      <x:c r="O188" s="129"/>
+      <x:c r="P188" s="129"/>
+      <x:c r="Q188" s="129"/>
+      <x:c r="R188" s="129"/>
+      <x:c r="S188" s="129"/>
+      <x:c r="T188" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH / ASSIGNED. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189">
+      <x:c r="A189" s="129" t="n">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="B189" s="129"/>
+      <x:c r="C189" s="129" t="str">
+        <x:v>complaints.view_reports</x:v>
+      </x:c>
+      <x:c r="D189" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E189" s="129" t="str">
+        <x:v>view</x:v>
+      </x:c>
+      <x:c r="F189" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G189" s="129"/>
+      <x:c r="H189" s="129"/>
+      <x:c r="I189" s="129"/>
+      <x:c r="J189" s="129"/>
+      <x:c r="K189" s="129"/>
+      <x:c r="L189" s="129"/>
+      <x:c r="M189" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N189" s="129"/>
+      <x:c r="O189" s="129"/>
+      <x:c r="P189" s="129"/>
+      <x:c r="Q189" s="129"/>
+      <x:c r="R189" s="129"/>
+      <x:c r="S189" s="129"/>
+      <x:c r="T189" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190">
+      <x:c r="A190" s="129" t="n">
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="B190" s="129"/>
+      <x:c r="C190" s="129" t="str">
+        <x:v>complaints.export</x:v>
+      </x:c>
+      <x:c r="D190" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E190" s="129" t="str">
+        <x:v>export</x:v>
+      </x:c>
+      <x:c r="F190" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G190" s="129"/>
+      <x:c r="H190" s="129"/>
+      <x:c r="I190" s="129"/>
+      <x:c r="J190" s="129"/>
+      <x:c r="K190" s="129"/>
+      <x:c r="L190" s="129"/>
+      <x:c r="M190" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N190" s="129"/>
+      <x:c r="O190" s="129"/>
+      <x:c r="P190" s="129"/>
+      <x:c r="Q190" s="129"/>
+      <x:c r="R190" s="129"/>
+      <x:c r="S190" s="129"/>
+      <x:c r="T190" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191">
+      <x:c r="A191" s="129" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="B191" s="129"/>
+      <x:c r="C191" s="129" t="str">
+        <x:v>complaints.link_requester</x:v>
+      </x:c>
+      <x:c r="D191" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E191" s="129" t="str">
+        <x:v>link_requester</x:v>
+      </x:c>
+      <x:c r="F191" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G191" s="129"/>
+      <x:c r="H191" s="129"/>
+      <x:c r="I191" s="129"/>
+      <x:c r="J191" s="129"/>
+      <x:c r="K191" s="129"/>
+      <x:c r="L191" s="129"/>
+      <x:c r="M191" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N191" s="129"/>
+      <x:c r="O191" s="129"/>
+      <x:c r="P191" s="129"/>
+      <x:c r="Q191" s="129"/>
+      <x:c r="R191" s="129"/>
+      <x:c r="S191" s="129"/>
+      <x:c r="T191" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192">
+      <x:c r="A192" s="129" t="n">
+        <x:v>191</x:v>
+      </x:c>
+      <x:c r="B192" s="129"/>
+      <x:c r="C192" s="129" t="str">
+        <x:v>complaints.link_visit</x:v>
+      </x:c>
+      <x:c r="D192" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E192" s="129" t="str">
+        <x:v>link_visit</x:v>
+      </x:c>
+      <x:c r="F192" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G192" s="129"/>
+      <x:c r="H192" s="129"/>
+      <x:c r="I192" s="129"/>
+      <x:c r="J192" s="129"/>
+      <x:c r="K192" s="129"/>
+      <x:c r="L192" s="129"/>
+      <x:c r="M192" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N192" s="129"/>
+      <x:c r="O192" s="129"/>
+      <x:c r="P192" s="129"/>
+      <x:c r="Q192" s="129"/>
+      <x:c r="R192" s="129"/>
+      <x:c r="S192" s="129"/>
+      <x:c r="T192" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH / ASSIGNED. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193">
+      <x:c r="A193" s="129" t="n">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="B193" s="129"/>
+      <x:c r="C193" s="129" t="str">
+        <x:v>complaints.link_device</x:v>
+      </x:c>
+      <x:c r="D193" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E193" s="129" t="str">
+        <x:v>link_device</x:v>
+      </x:c>
+      <x:c r="F193" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G193" s="129"/>
+      <x:c r="H193" s="129"/>
+      <x:c r="I193" s="129"/>
+      <x:c r="J193" s="129"/>
+      <x:c r="K193" s="129"/>
+      <x:c r="L193" s="129"/>
+      <x:c r="M193" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N193" s="129"/>
+      <x:c r="O193" s="129"/>
+      <x:c r="P193" s="129"/>
+      <x:c r="Q193" s="129"/>
+      <x:c r="R193" s="129"/>
+      <x:c r="S193" s="129"/>
+      <x:c r="T193" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH / ASSIGNED. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194">
+      <x:c r="A194" s="129" t="n">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="B194" s="129"/>
+      <x:c r="C194" s="129" t="str">
+        <x:v>complaints.link_target</x:v>
+      </x:c>
+      <x:c r="D194" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E194" s="129" t="str">
+        <x:v>link_target</x:v>
+      </x:c>
+      <x:c r="F194" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G194" s="129"/>
+      <x:c r="H194" s="129"/>
+      <x:c r="I194" s="129"/>
+      <x:c r="J194" s="129"/>
+      <x:c r="K194" s="129"/>
+      <x:c r="L194" s="129"/>
+      <x:c r="M194" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N194" s="129"/>
+      <x:c r="O194" s="129"/>
+      <x:c r="P194" s="129"/>
+      <x:c r="Q194" s="129"/>
+      <x:c r="R194" s="129"/>
+      <x:c r="S194" s="129"/>
+      <x:c r="T194" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH / ASSIGNED. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195">
+      <x:c r="A195" s="129" t="n">
+        <x:v>194</x:v>
+      </x:c>
+      <x:c r="B195" s="129"/>
+      <x:c r="C195" s="129" t="str">
+        <x:v>complaints.link_operational_work</x:v>
+      </x:c>
+      <x:c r="D195" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E195" s="129" t="str">
+        <x:v>link_work</x:v>
+      </x:c>
+      <x:c r="F195" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G195" s="129"/>
+      <x:c r="H195" s="129"/>
+      <x:c r="I195" s="129"/>
+      <x:c r="J195" s="129"/>
+      <x:c r="K195" s="129"/>
+      <x:c r="L195" s="129"/>
+      <x:c r="M195" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N195" s="129"/>
+      <x:c r="O195" s="129"/>
+      <x:c r="P195" s="129"/>
+      <x:c r="Q195" s="129"/>
+      <x:c r="R195" s="129"/>
+      <x:c r="S195" s="129"/>
+      <x:c r="T195" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL / BRANCH / ASSIGNED. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196">
+      <x:c r="A196" s="129" t="n">
+        <x:v>195</x:v>
+      </x:c>
+      <x:c r="B196" s="129"/>
+      <x:c r="C196" s="129" t="str">
+        <x:v>complaints.manage_duplicate_settings</x:v>
+      </x:c>
+      <x:c r="D196" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E196" s="129" t="str">
+        <x:v>duplicates</x:v>
+      </x:c>
+      <x:c r="F196" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G196" s="129"/>
+      <x:c r="H196" s="129"/>
+      <x:c r="I196" s="129"/>
+      <x:c r="J196" s="129"/>
+      <x:c r="K196" s="129"/>
+      <x:c r="L196" s="129"/>
+      <x:c r="M196" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N196" s="129"/>
+      <x:c r="O196" s="129"/>
+      <x:c r="P196" s="129"/>
+      <x:c r="Q196" s="129"/>
+      <x:c r="R196" s="129"/>
+      <x:c r="S196" s="129"/>
+      <x:c r="T196" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197">
+      <x:c r="A197" s="129" t="n">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="B197" s="129"/>
+      <x:c r="C197" s="129" t="str">
+        <x:v>complaints.manage_abuse_settings</x:v>
+      </x:c>
+      <x:c r="D197" s="129" t="str">
+        <x:v>الشكاوى</x:v>
+      </x:c>
+      <x:c r="E197" s="129" t="str">
+        <x:v>abuse</x:v>
+      </x:c>
+      <x:c r="F197" s="129" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G197" s="129"/>
+      <x:c r="H197" s="129"/>
+      <x:c r="I197" s="129"/>
+      <x:c r="J197" s="129"/>
+      <x:c r="K197" s="129"/>
+      <x:c r="L197" s="129"/>
+      <x:c r="M197" s="129" t="str">
+        <x:v>تُحدد حسب الدور</x:v>
+      </x:c>
+      <x:c r="N197" s="129"/>
+      <x:c r="O197" s="129"/>
+      <x:c r="P197" s="129"/>
+      <x:c r="Q197" s="129"/>
+      <x:c r="R197" s="129"/>
+      <x:c r="S197" s="129"/>
+      <x:c r="T197" s="129" t="str">
+        <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat: add operational reports and device lifecycle controls
</commit_message>
<xml_diff>
--- a/صلاحيات_النظام.xlsx
+++ b/صلاحيات_النظام.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="كل الصلاحيات" sheetId="1" r:id="R33547e2c24ea4a03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ملخص حسب الوحدة" sheetId="2" r:id="Rd0650eeff7cf438c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اختبار الأدوار" sheetId="3" r:id="R9d7cc976be6a4692"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اعتماد الزبائن" sheetId="4" r:id="R5a4a35e6dddb4789"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="كل الصلاحيات" sheetId="1" r:id="R132eb100e8464a47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ملخص حسب الوحدة" sheetId="2" r:id="R53a659fc806c4c65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اختبار الأدوار" sheetId="3" r:id="Rc0e728425657490b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اعتماد الزبائن" sheetId="4" r:id="R5132dac1913b47d7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -117,7 +117,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="44">
+  <x:fills count="47">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -334,8 +334,23 @@
         <x:fgColor rgb="FFC6EFCE"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC6EFCE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC6EFCE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC6EFCE"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="4">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -365,11 +380,25 @@
         <x:color rgb="FFBBF7D0"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9EAD3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9EAD3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9EAD3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9EAD3"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="131">
+  <x:cellXfs count="138">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -671,6 +700,17 @@
     <x:xf numFmtId="0" fontId="0" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="14" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="10" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="46" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -12359,6 +12399,206 @@
         <x:v>إضافة 2026-08-17: نطاق شكاوى مستقل؛ القرار الأمني يعتمد handlingBranchId وassignedUserId.</x:v>
       </x:c>
     </x:row>
+    <x:row r="211">
+      <x:c r="A211" s="133" t="n">
+        <x:v>210</x:v>
+      </x:c>
+      <x:c r="B211" s="133"/>
+      <x:c r="C211" s="133" t="str">
+        <x:v>التقارير</x:v>
+      </x:c>
+      <x:c r="D211" s="133" t="str">
+        <x:v>reports</x:v>
+      </x:c>
+      <x:c r="E211" s="133" t="str">
+        <x:v>work_files</x:v>
+      </x:c>
+      <x:c r="F211" s="133" t="str">
+        <x:v>view</x:v>
+      </x:c>
+      <x:c r="G211" s="133" t="str">
+        <x:v>عرض تقرير ملف العمل الجغرافي للمشرفات</x:v>
+      </x:c>
+      <x:c r="H211" s="133" t="str">
+        <x:v>reports.work_files.geo_supervisors.view</x:v>
+      </x:c>
+      <x:c r="I211" s="133" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J211" s="133" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="K211" s="133" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L211" s="133"/>
+      <x:c r="M211" s="133" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N211" s="133" t="str">
+        <x:v>إضافة 2026-08-25: صلاحية مستقلة للتقرير؛ النطاق يفرضه الخادم، والتصدير منفصل عن العرض.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212">
+      <x:c r="A212" s="133" t="n">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="B212" s="133"/>
+      <x:c r="C212" s="133" t="str">
+        <x:v>التقارير</x:v>
+      </x:c>
+      <x:c r="D212" s="133" t="str">
+        <x:v>reports</x:v>
+      </x:c>
+      <x:c r="E212" s="133" t="str">
+        <x:v>work_files</x:v>
+      </x:c>
+      <x:c r="F212" s="133" t="str">
+        <x:v>export</x:v>
+      </x:c>
+      <x:c r="G212" s="133" t="str">
+        <x:v>تصدير تقرير ملف العمل الجغرافي للمشرفات إلى Excel</x:v>
+      </x:c>
+      <x:c r="H212" s="133" t="str">
+        <x:v>reports.work_files.geo_supervisors.export</x:v>
+      </x:c>
+      <x:c r="I212" s="133" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J212" s="133" t="n">
+        <x:v>501</x:v>
+      </x:c>
+      <x:c r="K212" s="133" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L212" s="133"/>
+      <x:c r="M212" s="133" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N212" s="133" t="str">
+        <x:v>إضافة 2026-08-25: صلاحية مستقلة للتقرير؛ النطاق يفرضه الخادم، والتصدير منفصل عن العرض.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213">
+      <x:c r="A213" t="n">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="B213"/>
+      <x:c r="C213" t="str">
+        <x:v>التقارير</x:v>
+      </x:c>
+      <x:c r="D213" t="str">
+        <x:v>reports</x:v>
+      </x:c>
+      <x:c r="E213" t="str">
+        <x:v>daily_work</x:v>
+      </x:c>
+      <x:c r="F213" t="str">
+        <x:v>view</x:v>
+      </x:c>
+      <x:c r="G213" t="str">
+        <x:v>عرض تقرير سجل الزيارات اليومية</x:v>
+      </x:c>
+      <x:c r="H213" t="str">
+        <x:v>reports.daily_work.visits_log.view</x:v>
+      </x:c>
+      <x:c r="I213" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J213" t="n">
+        <x:v>510</x:v>
+      </x:c>
+      <x:c r="K213" t="str">
+        <x:v>✅</x:v>
+      </x:c>
+      <x:c r="L213"/>
+      <x:c r="M213" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N213" t="str">
+        <x:v>إضافة 2026-08-25: تقرير مستقل يُولّد يدويًا؛ النطاق يفرضه الخادم، والتصدير منفصل عن العرض.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214">
+      <x:c r="A214" t="n">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="B214"/>
+      <x:c r="C214" t="str">
+        <x:v>التقارير</x:v>
+      </x:c>
+      <x:c r="D214" t="str">
+        <x:v>reports</x:v>
+      </x:c>
+      <x:c r="E214" t="str">
+        <x:v>daily_work</x:v>
+      </x:c>
+      <x:c r="F214" t="str">
+        <x:v>export</x:v>
+      </x:c>
+      <x:c r="G214" t="str">
+        <x:v>تصدير تقرير سجل الزيارات اليومية إلى Excel</x:v>
+      </x:c>
+      <x:c r="H214" t="str">
+        <x:v>reports.daily_work.visits_log.export</x:v>
+      </x:c>
+      <x:c r="I214" t="str">
+        <x:v>عام (كل الفروع) / الفرع / المُسند فقط</x:v>
+      </x:c>
+      <x:c r="J214" t="n">
+        <x:v>511</x:v>
+      </x:c>
+      <x:c r="K214" t="str">
+        <x:v>✅</x:v>
+      </x:c>
+      <x:c r="L214"/>
+      <x:c r="M214" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N214" t="str">
+        <x:v>إضافة 2026-08-25: تقرير مستقل يُولّد يدويًا؛ النطاق يفرضه الخادم، والتصدير منفصل عن العرض.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215" ht="60" customHeight="1">
+      <x:c r="A215" s="137" t="n">
+        <x:v>214</x:v>
+      </x:c>
+      <x:c r="B215" s="137"/>
+      <x:c r="C215" s="137" t="str">
+        <x:v>الأجهزة</x:v>
+      </x:c>
+      <x:c r="D215" s="137" t="str">
+        <x:v>devices</x:v>
+      </x:c>
+      <x:c r="E215" s="137" t="str">
+        <x:v>installed_devices</x:v>
+      </x:c>
+      <x:c r="F215" s="137" t="str">
+        <x:v>delivery_suspension_manage</x:v>
+      </x:c>
+      <x:c r="G215" s="137" t="str">
+        <x:v>تعليق تسليم الجهاز وإعادته</x:v>
+      </x:c>
+      <x:c r="H215" s="137" t="str">
+        <x:v>installed_devices.delivery_suspension.manage</x:v>
+      </x:c>
+      <x:c r="I215" s="137" t="str">
+        <x:v>عام (كل الفروع) / الفرع</x:v>
+      </x:c>
+      <x:c r="J215" s="137" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="K215" s="137" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L215" s="137"/>
+      <x:c r="M215" s="137" t="str">
+        <x:v>الإضافة تمت</x:v>
+      </x:c>
+      <x:c r="N215" s="137" t="str">
+        <x:v>إضافة 2026-08-25: صلاحية مستقلة من تفاصيل الجهاز فقط؛ لا ترث منح contracts.edit، وتتحقق من فرع الجهاز وتسجل كل انتقال.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -12702,7 +12942,7 @@
         </x:is>
       </x:c>
       <x:c r="C22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -12772,12 +13012,23 @@
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" t="str">
+      <x:c r="A29" s="131" t="str">
+        <x:v>التقارير</x:v>
+      </x:c>
+      <x:c r="B29" s="131" t="str">
+        <x:v>reports</x:v>
+      </x:c>
+      <x:c r="C29" s="131" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
         <x:v>الإجمالي</x:v>
       </x:c>
-      <x:c r="B29"/>
-      <x:c r="C29" t="n">
-        <x:v>209</x:v>
+      <x:c r="B30"/>
+      <x:c r="C30" t="n">
+        <x:v>214</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -21545,6 +21796,238 @@
         <x:v>إضافة 2026-08-17. النطاقات المسموحة: GLOBAL. يجب اختبار فقد الصلاحية والفرع الخاطئ وعدم الإسناد والمسار GLOBAL.</x:v>
       </x:c>
     </x:row>
+    <x:row r="198">
+      <x:c r="A198" s="133" t="n">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="B198" s="133"/>
+      <x:c r="C198" s="133" t="str">
+        <x:v>reports.work_files.geo_supervisors.view</x:v>
+      </x:c>
+      <x:c r="D198" s="133" t="str">
+        <x:v>التقارير</x:v>
+      </x:c>
+      <x:c r="E198" s="133" t="str">
+        <x:v>view</x:v>
+      </x:c>
+      <x:c r="F198" s="133" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G198" s="133"/>
+      <x:c r="H198" s="133"/>
+      <x:c r="I198" s="133" t="str">
+        <x:v>✅</x:v>
+      </x:c>
+      <x:c r="J198" s="133" t="str">
+        <x:v>ASSIGNED</x:v>
+      </x:c>
+      <x:c r="K198" s="133" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L198" s="133"/>
+      <x:c r="M198" s="133" t="str">
+        <x:v>المشرفة تحصل على النطاق الشخصي افتراضيًا؛ بقية الأدوار تُحدد من إدارة الصلاحيات.</x:v>
+      </x:c>
+      <x:c r="N198" s="133"/>
+      <x:c r="O198" s="133"/>
+      <x:c r="P198" s="133"/>
+      <x:c r="Q198" s="133"/>
+      <x:c r="R198" s="133"/>
+      <x:c r="S198" s="133"/>
+      <x:c r="T198" s="133" t="str">
+        <x:v>اختبار إلزامي: فقد الصلاحية، فرع خاطئ، موظف آخر في ASSIGNED، BRANCH، GLOBAL، وفصل العرض عن التصدير.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199">
+      <x:c r="A199" s="133" t="n">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="B199" s="133"/>
+      <x:c r="C199" s="133" t="str">
+        <x:v>reports.work_files.geo_supervisors.export</x:v>
+      </x:c>
+      <x:c r="D199" s="133" t="str">
+        <x:v>التقارير</x:v>
+      </x:c>
+      <x:c r="E199" s="133" t="str">
+        <x:v>export</x:v>
+      </x:c>
+      <x:c r="F199" s="133" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G199" s="133"/>
+      <x:c r="H199" s="133"/>
+      <x:c r="I199" s="133" t="str">
+        <x:v>✅</x:v>
+      </x:c>
+      <x:c r="J199" s="133" t="str">
+        <x:v>ASSIGNED</x:v>
+      </x:c>
+      <x:c r="K199" s="133" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L199" s="133"/>
+      <x:c r="M199" s="133" t="str">
+        <x:v>المشرفة تحصل على النطاق الشخصي افتراضيًا؛ بقية الأدوار تُحدد من إدارة الصلاحيات.</x:v>
+      </x:c>
+      <x:c r="N199" s="133"/>
+      <x:c r="O199" s="133"/>
+      <x:c r="P199" s="133"/>
+      <x:c r="Q199" s="133"/>
+      <x:c r="R199" s="133"/>
+      <x:c r="S199" s="133"/>
+      <x:c r="T199" s="133" t="str">
+        <x:v>اختبار إلزامي: فقد الصلاحية، فرع خاطئ، موظف آخر في ASSIGNED، BRANCH، GLOBAL، وفصل العرض عن التصدير.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200">
+      <x:c r="A200" t="n">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="B200"/>
+      <x:c r="C200" t="str">
+        <x:v>reports.daily_work.visits_log.view</x:v>
+      </x:c>
+      <x:c r="D200" t="str">
+        <x:v>التقارير</x:v>
+      </x:c>
+      <x:c r="E200" t="str">
+        <x:v>view</x:v>
+      </x:c>
+      <x:c r="F200" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G200" t="str">
+        <x:v>✅</x:v>
+      </x:c>
+      <x:c r="H200" t="str">
+        <x:v>BRANCH</x:v>
+      </x:c>
+      <x:c r="I200" t="str">
+        <x:v>✅</x:v>
+      </x:c>
+      <x:c r="J200" t="str">
+        <x:v>ASSIGNED</x:v>
+      </x:c>
+      <x:c r="K200" t="str">
+        <x:v>✅</x:v>
+      </x:c>
+      <x:c r="L200" t="str">
+        <x:v>ASSIGNED</x:v>
+      </x:c>
+      <x:c r="M200" t="str">
+        <x:v>مدير الفرع ضمن فرعه، المشرفة والفني والمشرف ضمن الزيارات المرتبطة بهم، ومدير الشركة ضمن جميع الفروع.</x:v>
+      </x:c>
+      <x:c r="N200" t="str">
+        <x:v>✅</x:v>
+      </x:c>
+      <x:c r="O200" t="str">
+        <x:v>ASSIGNED</x:v>
+      </x:c>
+      <x:c r="P200"/>
+      <x:c r="Q200"/>
+      <x:c r="R200" t="str">
+        <x:v>✅</x:v>
+      </x:c>
+      <x:c r="S200" t="str">
+        <x:v>GLOBAL</x:v>
+      </x:c>
+      <x:c r="T200" t="str">
+        <x:v>اختبار إلزامي: فقد الصلاحية، فرع خاطئ، موظف آخر في ASSIGNED، BRANCH، GLOBAL، وفصل العرض عن التصدير.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201">
+      <x:c r="A201" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="B201"/>
+      <x:c r="C201" t="str">
+        <x:v>reports.daily_work.visits_log.export</x:v>
+      </x:c>
+      <x:c r="D201" t="str">
+        <x:v>التقارير</x:v>
+      </x:c>
+      <x:c r="E201" t="str">
+        <x:v>export</x:v>
+      </x:c>
+      <x:c r="F201" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G201" t="str">
+        <x:v>✅</x:v>
+      </x:c>
+      <x:c r="H201" t="str">
+        <x:v>BRANCH</x:v>
+      </x:c>
+      <x:c r="I201" t="str">
+        <x:v>✅</x:v>
+      </x:c>
+      <x:c r="J201" t="str">
+        <x:v>ASSIGNED</x:v>
+      </x:c>
+      <x:c r="K201" t="str">
+        <x:v>✅</x:v>
+      </x:c>
+      <x:c r="L201" t="str">
+        <x:v>ASSIGNED</x:v>
+      </x:c>
+      <x:c r="M201" t="str">
+        <x:v>مدير الفرع ضمن فرعه، المشرفة والفني والمشرف ضمن الزيارات المرتبطة بهم، ومدير الشركة ضمن جميع الفروع.</x:v>
+      </x:c>
+      <x:c r="N201" t="str">
+        <x:v>✅</x:v>
+      </x:c>
+      <x:c r="O201" t="str">
+        <x:v>ASSIGNED</x:v>
+      </x:c>
+      <x:c r="P201"/>
+      <x:c r="Q201"/>
+      <x:c r="R201" t="str">
+        <x:v>✅</x:v>
+      </x:c>
+      <x:c r="S201" t="str">
+        <x:v>GLOBAL</x:v>
+      </x:c>
+      <x:c r="T201" t="str">
+        <x:v>اختبار إلزامي: فقد الصلاحية، فرع خاطئ، موظف آخر في ASSIGNED، BRANCH، GLOBAL، وفصل العرض عن التصدير.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202" ht="54" customHeight="1">
+      <x:c r="A202" s="137" t="n">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="B202" s="137"/>
+      <x:c r="C202" s="137" t="str">
+        <x:v>installed_devices.delivery_suspension.manage</x:v>
+      </x:c>
+      <x:c r="D202" s="137" t="str">
+        <x:v>الأجهزة</x:v>
+      </x:c>
+      <x:c r="E202" s="137" t="str">
+        <x:v>delivery_suspension_manage</x:v>
+      </x:c>
+      <x:c r="F202" s="137" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="G202" s="137"/>
+      <x:c r="H202" s="137"/>
+      <x:c r="I202" s="137"/>
+      <x:c r="J202" s="137"/>
+      <x:c r="K202" s="137"/>
+      <x:c r="L202" s="137"/>
+      <x:c r="M202" s="137" t="str">
+        <x:v>تُحدد حسب الدور؛ لا توجد منحة baseline تلقائية.</x:v>
+      </x:c>
+      <x:c r="N202" s="137"/>
+      <x:c r="O202" s="137"/>
+      <x:c r="P202" s="137"/>
+      <x:c r="Q202" s="137"/>
+      <x:c r="R202" s="137"/>
+      <x:c r="S202" s="137"/>
+      <x:c r="T202" s="137" t="str">
+        <x:v>اختبار إلزامي: فقد الصلاحية، فرع خاطئ، BRANCH، GLOBAL، مسار super-admin، ومنع ASSIGNED. التعليق يلغي التسليم غير المنفذ ويرفض الزيارة التي بدأت.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>